<commit_message>
Update reports 2026-10-08 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-08.xlsx
+++ b/gex_pivot_levels_2026-10-08.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -544,12 +544,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$8.38M</t>
+          <t>-$9.07M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$12.65M</t>
+          <t>+$13.70M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -577,12 +577,12 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>-$1.99M</t>
+          <t>-$2.11M</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>+$6.39M</t>
+          <t>+$6.77M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-$21.64M</t>
+          <t>-$22.78M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$27.29M</t>
+          <t>+$28.73M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$176.01K</t>
+          <t>-$183.34K</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$17.28M</t>
+          <t>+$18.00M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -705,12 +705,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>-$16.42M</t>
+          <t>-$17.37M</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>+$32.97M</t>
+          <t>+$34.88M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -738,12 +738,12 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>-$3.41M</t>
+          <t>-$3.59M</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>+$9.81M</t>
+          <t>+$10.35M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -758,132 +758,128 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="5" t="n">
+        <v>7805.23</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7760</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>-$9.18M</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>+$16.29M</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
         <v>7815.23</v>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B10" s="2" t="n">
         <v>7770</v>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>-$19.31M</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>+$27.52M</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>-$20.20M</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>+$28.79M</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>7820.23</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B11" s="5" t="n">
         <v>7775</v>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>-$294.91K</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>+$24.31M</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>-$304.74K</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>+$25.12M</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
+    <row r="12">
+      <c r="A12" s="2" t="n">
         <v>7824.72</v>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B12" s="2" t="n">
         <v>775</v>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>-$13.72M</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>+$26.40M</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>7825.23</v>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>7780</v>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>-$14.03M</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>+$24.63M</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -891,101 +887,105 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
+        <v>7825.23</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>7780</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>-$14.33M</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>+$25.17M</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
         <v>7845.23</v>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B14" s="5" t="n">
         <v>7800</v>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>-$848.83K</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>+$39.72M</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>-$838.85K</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>+$39.26M</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="G14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
         <v>7870.23</v>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B15" s="2" t="n">
         <v>7825</v>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>+$15.48M</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>+$19.55M</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>+$14.34M</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>+$18.10M</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="n">
-        <v>7874.91</v>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>780</v>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>+$9.20M</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>+$29.35M</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>7884.94</v>
+        <v>7874.91</v>
       </c>
       <c r="B16" s="5" t="n">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
@@ -994,56 +994,85 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>+$11.40M</t>
+          <t>+$9.20M</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>+$23.90M</t>
+          <t>+$29.35M</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
+        <v>7884.94</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>781</v>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>+$11.40M</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>+$23.90M</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
         <v>7895.23</v>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B18" s="5" t="n">
         <v>7850</v>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>+$7.83M</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>+$12.86M</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>+$6.53M</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>+$10.71M</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G17"/>
+  <autoFilter ref="A1:G18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2971,7 +3000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3083,12 +3112,12 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>-$848.83K</t>
+          <t>-$838.85K</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>+$39.72M</t>
+          <t>+$39.26M</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -3117,12 +3146,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>-$16.42M</t>
+          <t>-$17.37M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>+$32.97M</t>
+          <t>+$34.88M</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3189,12 +3218,12 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>-$19.31M</t>
+          <t>-$20.20M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>+$27.52M</t>
+          <t>+$28.79M</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3227,12 +3256,12 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>-$21.64M</t>
+          <t>-$22.78M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>+$27.29M</t>
+          <t>+$28.73M</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -3341,12 +3370,12 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>-$14.03M</t>
+          <t>-$14.33M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>+$24.63M</t>
+          <t>+$25.17M</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -3379,12 +3408,12 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>-$294.91K</t>
+          <t>-$304.74K</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>+$24.31M</t>
+          <t>+$25.12M</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -3493,12 +3522,12 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>+$15.48M</t>
+          <t>+$14.34M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>+$19.55M</t>
+          <t>+$18.10M</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -3531,12 +3560,12 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>-$176.01K</t>
+          <t>-$183.34K</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>+$17.28M</t>
+          <t>+$18.00M</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -3551,148 +3580,148 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7805.23</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>7760</v>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>-$9.18M</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>+$16.29M</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>4284.05</v>
       </c>
-      <c r="C16" s="2" t="n">
+      <c r="C17" s="2" t="n">
         <v>88</v>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>+$13.20M</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>+$14.59M</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B18" s="2" t="n">
+        <v>7745.23</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>7700</v>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>-$9.07M</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>+$13.70M</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
         <v>7774.53</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C19" s="5" t="n">
         <v>770</v>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>-$3.98M</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>+$13.17M</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="n">
-        <v>7895.23</v>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>7850</v>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>+$7.83M</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>+$12.86M</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>7745.23</v>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>7700</v>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>-$8.38M</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>+$12.65M</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -3777,222 +3806,218 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
+        <v>7895.23</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>7850</v>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>+$6.53M</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>+$10.71M</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
         <v>7800.23</v>
       </c>
-      <c r="C22" s="5" t="n">
+      <c r="C23" s="5" t="n">
         <v>7755</v>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>-$3.41M</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>+$9.81M</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>-$3.59M</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>+$10.35M</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>4138.01</v>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>-$8.02M</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>+$8.71M</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>4138.01</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>-$8.02M</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>+$8.71M</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B25" s="2" t="n">
         <v>2756.44</v>
       </c>
-      <c r="C24" s="2" t="n">
+      <c r="C25" s="2" t="n">
         <v>274</v>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>-$7.19M</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>+$7.36M</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>7760.23</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>7715</v>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>-$1.99M</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>+$6.39M</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>7760.23</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>7715</v>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>-$2.11M</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>+$6.77M</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n">
+      <c r="B27" s="5" t="n">
         <v>31041.12</v>
       </c>
-      <c r="C26" s="5" t="n">
+      <c r="C27" s="5" t="n">
         <v>750</v>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>-$1.41M</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>+$4.98M</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>4357.08</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>89.5</v>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>+$4.89M</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>+$4.96M</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4001,28 +4026,28 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>89.93000000000001</v>
+        <v>4357.08</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>144</v>
+        <v>89.5</v>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>+$2.69M</t>
+          <t>+$4.89M</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>+$4.89M</t>
+          <t>+$4.96M</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -4039,150 +4064,150 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>89.93000000000001</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>+$2.69M</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>+$4.89M</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B30" s="2" t="n">
         <v>4150.66</v>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C30" s="2" t="n">
         <v>375</v>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>-$3.59M</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>+$4.30M</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>2786.62</v>
-      </c>
-      <c r="C30" s="5" t="n">
-        <v>277</v>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>-$2.02M</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>+$3.57M</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>2786.62</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>277</v>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>-$2.02M</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>+$3.57M</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B31" s="5" t="n">
+      <c r="B32" s="5" t="n">
         <v>3991.96</v>
       </c>
-      <c r="C31" s="5" t="n">
+      <c r="C32" s="5" t="n">
         <v>82</v>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E32" s="7" t="inlineStr">
         <is>
           <t>-$3.44M</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>+$3.44M</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>86.8</v>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>139</v>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>-$3.35M</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>+$3.41M</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -4191,96 +4216,100 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
+        <v>86.8</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>-$3.35M</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>+$3.41M</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
         <v>92.42</v>
       </c>
-      <c r="C33" s="2" t="n">
+      <c r="C34" s="2" t="n">
         <v>148</v>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>+$2.47M</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>+$3.20M</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="n">
-        <v>4478.78</v>
-      </c>
-      <c r="C34" s="5" t="n">
-        <v>92</v>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>+$1.75M</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>+$1.79M</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>93.67</v>
+        <v>4478.78</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>150</v>
+        <v>92</v>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>GDX</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>+$935.80K</t>
+          <t>+$1.75M</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>+$1.58M</t>
+          <t>+$1.79M</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -4297,10 +4326,10 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>94.3</v>
+        <v>93.67</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
@@ -4309,24 +4338,20 @@
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>+$1.18M</t>
+          <t>+$935.80K</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>+$1.47M</t>
+          <t>+$1.58M</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H36" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -4335,104 +4360,108 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
+        <v>94.3</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>151</v>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>+$1.18M</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>+$1.47M</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
         <v>89.3</v>
       </c>
-      <c r="C37" s="5" t="n">
+      <c r="C38" s="5" t="n">
         <v>143</v>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E38" s="7" t="inlineStr">
         <is>
           <t>-$916.40K</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>+$1.32M</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
+      <c r="B39" s="2" t="n">
         <v>84.31</v>
       </c>
-      <c r="C38" s="2" t="n">
+      <c r="C39" s="2" t="n">
         <v>135</v>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>-$1.28M</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>+$1.32M</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="n">
-        <v>2615.6</v>
-      </c>
-      <c r="C39" s="5" t="n">
-        <v>260</v>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>-$1.23M</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
-          <t>+$1.23M</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -4441,10 +4470,10 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>2686.02</v>
+        <v>2615.6</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
@@ -4453,12 +4482,12 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>-$1.11M</t>
+          <t>-$1.23M</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>+$1.11M</t>
+          <t>+$1.23M</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -4471,40 +4500,36 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>4183.86</v>
+        <v>2686.02</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>378</v>
+        <v>267</v>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>-$685.42K</t>
+          <t>-$1.11M</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>+$1.07M</t>
+          <t>+$1.11M</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -4513,110 +4538,110 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
+        <v>4183.86</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>378</v>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>-$685.42K</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>+$1.07M</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
         <v>4161.73</v>
       </c>
-      <c r="C42" s="5" t="n">
+      <c r="C43" s="5" t="n">
         <v>376</v>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E42" s="9" t="inlineStr">
+      <c r="E43" s="9" t="inlineStr">
         <is>
           <t>+$67.03K</t>
         </is>
       </c>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>+$981.88K</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B44" s="2" t="n">
         <v>31423.92</v>
       </c>
-      <c r="C43" s="2" t="n">
+      <c r="C44" s="2" t="n">
         <v>31225</v>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E43" s="8" t="inlineStr">
+      <c r="E44" s="8" t="inlineStr">
         <is>
           <t>+$683.34K</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F44" s="3" t="inlineStr">
         <is>
           <t>+$715.12K</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G44" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr">
+      <c r="H44" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="n">
-        <v>91.18000000000001</v>
-      </c>
-      <c r="C44" s="5" t="n">
-        <v>146</v>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="inlineStr">
-        <is>
-          <t>-$9.08K</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="inlineStr">
-        <is>
-          <t>+$671.93K</t>
-        </is>
-      </c>
-      <c r="G44" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4627,24 +4652,24 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>93.05</v>
+        <v>91.18000000000001</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E45" s="9" t="inlineStr">
-        <is>
-          <t>+$185.55K</t>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>-$9.08K</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>+$546.75K</t>
+          <t>+$671.93K</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -4665,58 +4690,62 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>81.18000000000001</v>
+        <v>93.05</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E46" s="7" t="inlineStr">
-        <is>
-          <t>-$502.83K</t>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>+$185.55K</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>+$543.39K</t>
+          <t>+$546.75K</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H46" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>4039.98</v>
+        <v>81.18000000000001</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>365</v>
+        <v>130</v>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>-$451.30K</t>
+          <t>-$502.83K</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>+$460.42K</t>
+          <t>+$543.39K</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
@@ -4733,72 +4762,68 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
+        <v>4039.98</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>365</v>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>-$451.30K</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>+$460.42K</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
         <v>4308.39</v>
       </c>
-      <c r="C48" s="5" t="n">
+      <c r="C49" s="5" t="n">
         <v>88.5</v>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E48" s="9" t="inlineStr">
+      <c r="E49" s="9" t="inlineStr">
         <is>
           <t>+$219.83K</t>
         </is>
       </c>
-      <c r="F48" s="6" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>+$337.23K</t>
         </is>
       </c>
-      <c r="G48" s="6" t="inlineStr">
+      <c r="G49" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H48" s="6" t="inlineStr">
+      <c r="H49" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="n">
-        <v>31358.92</v>
-      </c>
-      <c r="C49" s="2" t="n">
-        <v>31160</v>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>+$201.92K</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>+$336.53K</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H49" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4809,10 +4834,10 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>31548.92</v>
+        <v>31358.92</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>31350</v>
+        <v>31160</v>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
@@ -4821,12 +4846,12 @@
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>+$243.05K</t>
+          <t>+$201.92K</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>+$307.86K</t>
+          <t>+$336.53K</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -4847,10 +4872,10 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>31198.92</v>
+        <v>31548.92</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>31000</v>
+        <v>31350</v>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
@@ -4859,12 +4884,12 @@
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>+$28.36K</t>
+          <t>+$243.05K</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>+$247.10K</t>
+          <t>+$307.86K</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -4885,100 +4910,100 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
+        <v>31198.92</v>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>31000</v>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>+$28.36K</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>+$247.10K</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
         <v>31298.92</v>
       </c>
-      <c r="C52" s="2" t="n">
+      <c r="C53" s="2" t="n">
         <v>31100</v>
       </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E52" s="8" t="inlineStr">
+      <c r="E53" s="8" t="inlineStr">
         <is>
           <t>+$105.94K</t>
         </is>
       </c>
-      <c r="F52" s="3" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>+$243.67K</t>
         </is>
       </c>
-      <c r="G52" s="3" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H52" s="3" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n">
-        <v>31338.92</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>31140</v>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>-$56.09K</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
-          <t>+$224.35K</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>84.93000000000001</v>
+        <v>31338.92</v>
       </c>
       <c r="C54" s="5" t="n">
-        <v>136</v>
+        <v>31140</v>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>-$205.79K</t>
+          <t>-$56.09K</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>+$215.15K</t>
+          <t>+$224.35K</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
@@ -4988,35 +5013,35 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>31308.92</v>
+        <v>84.93000000000001</v>
       </c>
       <c r="C55" s="5" t="n">
-        <v>31110</v>
+        <v>136</v>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>-$116.54K</t>
+          <t>-$205.79K</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>+$201.29K</t>
+          <t>+$215.15K</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
@@ -5026,7 +5051,7 @@
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -5037,184 +5062,188 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
+        <v>31308.92</v>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>31110</v>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>-$116.54K</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>+$201.29K</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
         <v>31328.92</v>
       </c>
-      <c r="C56" s="5" t="n">
+      <c r="C57" s="5" t="n">
         <v>31130</v>
       </c>
-      <c r="D56" s="6" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E56" s="9" t="inlineStr">
+      <c r="E57" s="9" t="inlineStr">
         <is>
           <t>+$95.35K</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>+$196.31K</t>
         </is>
       </c>
-      <c r="G56" s="6" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H56" s="6" t="inlineStr">
+      <c r="H57" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B57" s="2" t="n">
+      <c r="B58" s="2" t="n">
         <v>31248.92</v>
       </c>
-      <c r="C57" s="2" t="n">
+      <c r="C58" s="2" t="n">
         <v>31050</v>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="E58" s="4" t="inlineStr">
         <is>
           <t>-$135.55K</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
+      <c r="F58" s="3" t="inlineStr">
         <is>
           <t>+$191.63K</t>
         </is>
       </c>
-      <c r="G57" s="3" t="inlineStr">
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H57" s="3" t="inlineStr">
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B58" s="5" t="n">
+      <c r="B59" s="5" t="n">
         <v>31368.92</v>
       </c>
-      <c r="C58" s="5" t="n">
+      <c r="C59" s="5" t="n">
         <v>31170</v>
       </c>
-      <c r="D58" s="6" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E58" s="9" t="inlineStr">
+      <c r="E59" s="9" t="inlineStr">
         <is>
           <t>+$22.44K</t>
         </is>
       </c>
-      <c r="F58" s="6" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>+$190.70K</t>
         </is>
       </c>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H58" s="6" t="inlineStr">
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B59" s="2" t="n">
+      <c r="B60" s="2" t="n">
         <v>31378.92</v>
       </c>
-      <c r="C59" s="2" t="n">
+      <c r="C60" s="2" t="n">
         <v>31180</v>
       </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E59" s="8" t="inlineStr">
+      <c r="E60" s="8" t="inlineStr">
         <is>
           <t>+$145.83K</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr">
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>+$179.48K</t>
         </is>
       </c>
-      <c r="G59" s="3" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H59" s="3" t="inlineStr">
+      <c r="H60" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="n">
-        <v>31498.92</v>
-      </c>
-      <c r="C60" s="5" t="n">
-        <v>31300</v>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E60" s="9" t="inlineStr">
-        <is>
-          <t>+$135.55K</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>+$172.94K</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
@@ -5223,10 +5252,10 @@
         </is>
       </c>
       <c r="B61" s="5" t="n">
-        <v>31408.92</v>
+        <v>31498.92</v>
       </c>
       <c r="C61" s="5" t="n">
-        <v>31210</v>
+        <v>31300</v>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
@@ -5235,24 +5264,20 @@
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>+$162.66K</t>
+          <t>+$135.55K</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>+$162.66K</t>
+          <t>+$172.94K</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H61" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
@@ -5261,104 +5286,108 @@
         </is>
       </c>
       <c r="B62" s="5" t="n">
+        <v>31408.92</v>
+      </c>
+      <c r="C62" s="5" t="n">
+        <v>31210</v>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>+$162.66K</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>+$162.66K</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n">
         <v>31278.92</v>
       </c>
-      <c r="C62" s="5" t="n">
+      <c r="C63" s="5" t="n">
         <v>31080</v>
       </c>
-      <c r="D62" s="6" t="inlineStr">
+      <c r="D63" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E62" s="7" t="inlineStr">
+      <c r="E63" s="7" t="inlineStr">
         <is>
           <t>-$99.71K</t>
         </is>
       </c>
-      <c r="F62" s="6" t="inlineStr">
+      <c r="F63" s="6" t="inlineStr">
         <is>
           <t>+$159.54K</t>
         </is>
       </c>
-      <c r="G62" s="6" t="inlineStr">
+      <c r="G63" s="6" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H62" s="6" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
+      <c r="H63" s="6" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B63" s="2" t="n">
+      <c r="B64" s="2" t="n">
         <v>31518.92</v>
       </c>
-      <c r="C63" s="2" t="n">
+      <c r="C64" s="2" t="n">
         <v>31320</v>
       </c>
-      <c r="D63" s="3" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E63" s="8" t="inlineStr">
+      <c r="E64" s="8" t="inlineStr">
         <is>
           <t>+$143.96K</t>
         </is>
       </c>
-      <c r="F63" s="3" t="inlineStr">
+      <c r="F64" s="3" t="inlineStr">
         <is>
           <t>+$143.96K</t>
         </is>
       </c>
-      <c r="G63" s="3" t="inlineStr">
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H63" s="3" t="inlineStr">
+      <c r="H64" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="n">
-        <v>31448.92</v>
-      </c>
-      <c r="C64" s="5" t="n">
-        <v>31250</v>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E64" s="9" t="inlineStr">
-        <is>
-          <t>+$90.05K</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>+$143.02K</t>
-        </is>
-      </c>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
@@ -5367,10 +5396,10 @@
         </is>
       </c>
       <c r="B65" s="5" t="n">
-        <v>31418.92</v>
+        <v>31448.92</v>
       </c>
       <c r="C65" s="5" t="n">
-        <v>31220</v>
+        <v>31250</v>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
@@ -5379,24 +5408,20 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>+$5.61K</t>
+          <t>+$90.05K</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>+$129.00K</t>
+          <t>+$143.02K</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H65" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
@@ -5405,10 +5430,10 @@
         </is>
       </c>
       <c r="B66" s="5" t="n">
-        <v>31528.92</v>
+        <v>31418.92</v>
       </c>
       <c r="C66" s="5" t="n">
-        <v>31330</v>
+        <v>31220</v>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
@@ -5417,20 +5442,24 @@
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>+$30.54K</t>
+          <t>+$5.61K</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>+$91.61K</t>
+          <t>+$129.00K</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H66" s="6" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
@@ -5439,36 +5468,32 @@
         </is>
       </c>
       <c r="B67" s="5" t="n">
-        <v>31468.92</v>
+        <v>31528.92</v>
       </c>
       <c r="C67" s="5" t="n">
-        <v>31270</v>
+        <v>31330</v>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E67" s="7" t="inlineStr">
-        <is>
-          <t>-$29.91K</t>
+      <c r="E67" s="9" t="inlineStr">
+        <is>
+          <t>+$30.54K</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>+$79.77K</t>
+          <t>+$91.61K</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H67" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -5477,10 +5502,10 @@
         </is>
       </c>
       <c r="B68" s="5" t="n">
-        <v>31388.92</v>
+        <v>31468.92</v>
       </c>
       <c r="C68" s="5" t="n">
-        <v>31190</v>
+        <v>31270</v>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
@@ -5489,12 +5514,12 @@
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>-$5.61K</t>
+          <t>-$29.91K</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>+$61.70K</t>
+          <t>+$79.77K</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr">
@@ -5515,39 +5540,77 @@
         </is>
       </c>
       <c r="B69" s="5" t="n">
+        <v>31388.92</v>
+      </c>
+      <c r="C69" s="5" t="n">
+        <v>31190</v>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>-$5.61K</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>+$61.70K</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="n">
         <v>31523.92</v>
       </c>
-      <c r="C69" s="5" t="n">
+      <c r="C70" s="5" t="n">
         <v>31325</v>
       </c>
-      <c r="D69" s="6" t="inlineStr">
+      <c r="D70" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E69" s="9" t="inlineStr">
+      <c r="E70" s="9" t="inlineStr">
         <is>
           <t>+$17.45K</t>
         </is>
       </c>
-      <c r="F69" s="6" t="inlineStr">
+      <c r="F70" s="6" t="inlineStr">
         <is>
           <t>+$26.17K</t>
         </is>
       </c>
-      <c r="G69" s="6" t="inlineStr">
+      <c r="G70" s="6" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H69" s="6" t="inlineStr">
+      <c r="H70" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H69"/>
+  <autoFilter ref="A1:H70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>